<commit_message>
The app starts from Adam, using the README.md plus setup_notes.md
</commit_message>
<xml_diff>
--- a/bots/conversation_store.xlsx
+++ b/bots/conversation_store.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sessions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sessions" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E128"/>
+  <dimension ref="A1:E130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
@@ -6874,6 +6874,72 @@
         </is>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>0122f583-7231-45ba-8f84-075e5f4a460a</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>user: Are you working?
+assistant: Hello! I'm here to help you set up reminders. What would you like to be reminded about?
+user: Remind me to take out the trash after lunch
+assistant: Great! I'll set up a reminder for you to take out the trash after lunch. 
+Would you like this reminder to be for today, tomorrow, or a specific date? Also, should it repeat daily, weekly, or just once?
+user: Repeat it daily
+assistant: Perfect! I'll set up a daily reminder for you to take out the trash after lunch. Is there a specific time you'd like me to set for "after lunch," or should I leave it open-ended?</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>3589071e-dd20-4fae-a014-6aaad301d227</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>user: please remind me to take out the trash after lunch
+assistant: Great! I'll set up a reminder for you to take out the trash after lunch. Would you like this reminder to be for today, or would you like it to repeat on certain days?
+user: every day
+assistant: Thank you for the information! I'll set up a daily reminder for you to take out the trash after lunch. If there's anything else you need, feel free to let me know. [ChatEnded]
+user: every day
+assistant: It looks like you've already set up a daily reminder to take out the trash after lunch. If there's anything else you need help with, feel free to let me know!</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>{
+  "content": {
+    "task": "Take out the trash",
+    "date": "today",
+    "time": {
+      "exact_time": {
+        "start_time": "13:00",
+        "end_time": "14:00"
+      },
+      "time_inferred": "after lunch"
+    },
+    "recurrence": {
+      "type": "daily",
+      "details": {
+        "days": null,
+        "occurrence_frequency": "once"
+      }
+    },
+    "priority": "medium"
+  }
+}</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>def reminder_c384b472_0776_4be8_8301_7c9b7af929ca(time=None, activity_data=None, sensor_data=None, blackboard=None):
+    return activity_data.get('activity') == "Eating" and activity_data.get('status') == "end"</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add writing conversation.txt and prompt.txt to bots/ for debugging chatgpt (gpt api)
</commit_message>
<xml_diff>
--- a/bots/conversation_store.xlsx
+++ b/bots/conversation_store.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E131"/>
+  <dimension ref="A1:E134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
@@ -6991,6 +6991,113 @@
         </is>
       </c>
     </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>0c3327d3-7342-47f3-b3c5-a6b276e87233</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>user: remind me to eat after I wake up
+assistant: Great! I'll set up a reminder for you to eat after you wake up. Would you like this reminder to repeat every day, or just once?
+user: every day
+assistant: Thank you for the information! I'll set up a daily reminder for you to eat after you wake up. If there's anything else you need, feel free to let me know. [ChatEnded]</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>{
+  "content": {
+    "task": "Eat after I wake up",
+    "date": "today",
+    "time": {
+      "exact_time": {
+        "start_time": null,
+        "end_time": null
+      },
+      "time_inferred": "after I wake up"
+    },
+    "recurrence": {
+      "type": "daily",
+      "details": {
+        "days": null,
+        "occurrence_frequency": "once"
+      }
+    },
+    "priority": "medium"
+  }
+}</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>def reminder_ad765cf2_8340_47a9_9902_216a1abd5384(time=None, activity_data=None, sensor_data=None, blackboard=None):
+    return activity_data.get('activity') == "Sleeping" and activity_data.get('status') == "end"</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>677bea34-81dc-49a7-af24-2ca3f093b7f1</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>user: I want to go eat banana after dinner
+assistant: Great! I can help you set a reminder for that. 
+1. **Time/Event**: When would you like to be reminded? For example, "Remind me right after dinner" or "Remind me at 8:00 PM."
+2. **Date (Optional)**: Would you like this reminder for today, tomorrow, or a specific date?
+3. **Recurrence**: Should this reminder repeat, or is it just for one time?
+Let me know these details, and I'll set up the reminder for you!</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>789c9091-8112-449c-9586-59fe1d5ef8e9</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>user: Please remind me to watch tv after dinner
+assistant: Great! I'll set up a reminder for you to watch TV after dinner. Would you like this reminder for today, or would you prefer a specific date? Also, should this reminder repeat, or would you like it just once?</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>{
+  "content": {
+    "task": "Bring in my cactus",
+    "date": "today",
+    "time": {
+      "exact_time": {
+        "start_time": null,
+        "end_time": null
+      },
+      "time_inferred": "when it starts raining"
+    },
+    "recurrence": {
+      "type": "daily",
+      "details": {
+        "days": null,
+        "occurrence_frequency": "once"
+      }
+    },
+    "priority": "medium"
+  }
+}</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>def reminder_55146fe5_00eb_4e89_a608_45ad3722e967(time=None, activity_data=None, sensor_data=None, blackboard=None):
+    return sensor_data.get('rain_sensor', {}).get('status', False)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>